<commit_message>
backend package refactor and community feature
</commit_message>
<xml_diff>
--- a/DB산출물/04_테이블정의서.xlsx
+++ b/DB산출물/04_테이블정의서.xlsx
@@ -5,16 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pknu_202601\day69-day74_미니프로젝트(2차)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\pknu_202601\day69-day74_미니프로젝트(2차)\project2\DB산출물\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88A94BC-989F-4A1F-8641-CE3AB93C89BC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{834AFB55-E511-4A7E-9FFA-6107B19D6C0A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12060" activeTab="2" xr2:uid="{7B4FFD32-6000-4470-9C7F-42EB358F027C}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12060" xr2:uid="{7B4FFD32-6000-4470-9C7F-42EB358F027C}"/>
   </bookViews>
   <sheets>
     <sheet name="Member" sheetId="1" r:id="rId1"/>
-    <sheet name="Health Diagnose" sheetId="2" r:id="rId2"/>
+    <sheet name="Data" sheetId="2" r:id="rId2"/>
     <sheet name="Community" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="133">
   <si>
     <t>테이블정의서</t>
   </si>
@@ -96,10 +96,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>MEM_HO_LNCM</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>MEM_CREATED</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -187,14 +183,6 @@
   </si>
   <si>
     <t>회원정보</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>건강진단정보</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>DIAGNOSIS_ID</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -423,14 +411,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>HEALTH DIAGNOSE</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>회원의 건강검진 결과와 생활습관 정보를 저장하는 엔터티</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>회원정보를 저장 관리하기 위한 엔터티</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -515,6 +495,38 @@
   </si>
   <si>
     <t>NOT NULL</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DATA_ID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>predict</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>예측결과</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NUMBER(5,4)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>DATA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>회원의 건강정보와 생활습관을 저장하는 엔터티</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>정보</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1 : 남, 2 : 여</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -811,7 +823,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -839,24 +851,33 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -884,42 +905,42 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -935,14 +956,8 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1258,7 +1273,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB060BAC-2233-45AD-9EBA-22CADB6F76BA}">
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1274,93 +1289,93 @@
   <sheetData>
     <row r="1" spans="1:10" ht="16.5" customHeight="1"/>
     <row r="2" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="22" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="20" t="s">
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22" t="s">
+      <c r="H4" s="24"/>
+      <c r="I4" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="21"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="13" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="18" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="15" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="14"/>
+      <c r="J5" s="16"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="18"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="21"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>8</v>
@@ -1374,12 +1389,12 @@
       <c r="F7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="12"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="3">
@@ -1389,21 +1404,21 @@
         <v>15</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
+        <v>41</v>
+      </c>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="3">
@@ -1413,19 +1428,19 @@
         <v>16</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F9" s="3"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="3">
@@ -1435,19 +1450,19 @@
         <v>17</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F10" s="3"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="9"/>
-      <c r="J10" s="9"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="17"/>
+      <c r="I10" s="17"/>
+      <c r="J10" s="17"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="3">
@@ -1457,17 +1472,17 @@
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="17"/>
+      <c r="J11" s="17"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="3">
@@ -1477,17 +1492,17 @@
         <v>19</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="17"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="17"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3">
@@ -1504,45 +1519,25 @@
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="17"/>
+      <c r="I13" s="17"/>
+      <c r="J13" s="17"/>
     </row>
     <row r="14" spans="1:10">
-      <c r="A14" s="3">
-        <v>8</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+      <c r="A14" s="1"/>
+      <c r="B14" s="1"/>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
+      <c r="F14" s="1"/>
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="18">
     <mergeCell ref="A2:J3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:F4"/>
@@ -1551,7 +1546,6 @@
     <mergeCell ref="G7:J7"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="G13:J13"/>
-    <mergeCell ref="G14:J14"/>
     <mergeCell ref="C5:F5"/>
     <mergeCell ref="G5:H5"/>
     <mergeCell ref="I5:J5"/>
@@ -1571,7 +1565,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16AE0AA4-CB13-4D0B-9558-40535FA8F1BE}">
-  <dimension ref="A2:J34"/>
+  <dimension ref="A2:J35"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="14.375" bestFit="1" customWidth="1"/>
@@ -1584,93 +1578,93 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="22" t="s">
-        <v>106</v>
-      </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="20" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22" t="s">
+      <c r="H4" s="24"/>
+      <c r="I4" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="21"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="13" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="18" t="s">
+        <v>131</v>
+      </c>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="15" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="14"/>
+      <c r="J5" s="16"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" s="17"/>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="18"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="18" t="s">
+        <v>130</v>
+      </c>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="20"/>
+      <c r="J6" s="21"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>8</v>
@@ -1684,36 +1678,36 @@
       <c r="F7" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="11"/>
-      <c r="I7" s="11"/>
-      <c r="J7" s="12"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="14"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="3">
         <v>1</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>125</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="9"/>
-      <c r="J8" s="9"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
     </row>
     <row r="9" spans="1:10" ht="17.25">
       <c r="A9" s="3">
@@ -1723,518 +1717,541 @@
         <v>15</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="9"/>
-      <c r="J9" s="9"/>
+        <v>44</v>
+      </c>
+      <c r="G9" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="H9" s="17"/>
+      <c r="I9" s="17"/>
+      <c r="J9" s="17"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="3">
         <v>3</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E10" s="3"/>
       <c r="F10" s="3"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="11" spans="1:10" ht="17.25">
       <c r="A11" s="3">
         <v>4</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E11" s="3"/>
       <c r="F11" s="3"/>
-      <c r="G11" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="27"/>
+      <c r="G11" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="3">
         <v>5</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="27"/>
+      <c r="G12" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="29"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="3">
         <v>6</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="27"/>
+      <c r="G13" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="29"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="3">
         <v>7</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
-      <c r="G14" s="25" t="s">
-        <v>62</v>
-      </c>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="27"/>
+      <c r="G14" s="27" t="s">
+        <v>59</v>
+      </c>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="29"/>
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="3">
         <v>8</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
-      <c r="G15" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="H15" s="31"/>
-      <c r="I15" s="31"/>
-      <c r="J15" s="32"/>
+      <c r="G15" s="31" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" s="32"/>
+      <c r="I15" s="32"/>
+      <c r="J15" s="33"/>
     </row>
     <row r="16" spans="1:10" ht="17.25">
       <c r="A16" s="3">
         <v>9</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="26"/>
-      <c r="I16" s="26"/>
-      <c r="J16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="28"/>
+      <c r="I16" s="28"/>
+      <c r="J16" s="29"/>
     </row>
     <row r="17" spans="1:10" ht="17.25">
       <c r="A17" s="3">
         <v>10</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="26"/>
-      <c r="I17" s="26"/>
-      <c r="J17" s="27"/>
+      <c r="G17" s="27"/>
+      <c r="H17" s="28"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="29"/>
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="3">
         <v>11</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="26"/>
-      <c r="I18" s="26"/>
-      <c r="J18" s="27"/>
+      <c r="G18" s="27"/>
+      <c r="H18" s="28"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="29"/>
     </row>
     <row r="19" spans="1:10" ht="17.25">
       <c r="A19" s="3">
         <v>12</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="26"/>
-      <c r="I19" s="26"/>
-      <c r="J19" s="27"/>
+      <c r="G19" s="27"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="29"/>
     </row>
     <row r="20" spans="1:10" ht="17.25">
       <c r="A20" s="3">
         <v>13</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="E20" s="3"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="26"/>
-      <c r="I20" s="26"/>
-      <c r="J20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="28"/>
+      <c r="I20" s="28"/>
+      <c r="J20" s="29"/>
     </row>
     <row r="21" spans="1:10" ht="17.25">
       <c r="A21" s="3">
         <v>14</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="26"/>
-      <c r="I21" s="26"/>
-      <c r="J21" s="27"/>
+      <c r="G21" s="27"/>
+      <c r="H21" s="28"/>
+      <c r="I21" s="28"/>
+      <c r="J21" s="29"/>
     </row>
     <row r="22" spans="1:10" ht="17.25">
       <c r="A22" s="7">
         <v>15</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
-      <c r="G22" s="33" t="s">
-        <v>94</v>
-      </c>
-      <c r="H22" s="34"/>
-      <c r="I22" s="34"/>
-      <c r="J22" s="35"/>
+      <c r="G22" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="H22" s="35"/>
+      <c r="I22" s="35"/>
+      <c r="J22" s="36"/>
     </row>
     <row r="23" spans="1:10" ht="17.25" customHeight="1">
-      <c r="A23" s="9">
+      <c r="A23" s="17">
         <v>16</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="D23" s="29" t="s">
+      <c r="B23" s="17" t="s">
         <v>92</v>
       </c>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-      <c r="G23" s="28" t="s">
-        <v>100</v>
-      </c>
-      <c r="H23" s="28"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="28"/>
+      <c r="C23" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="30" t="s">
+        <v>89</v>
+      </c>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="H23" s="37"/>
+      <c r="I23" s="37"/>
+      <c r="J23" s="37"/>
     </row>
     <row r="24" spans="1:10">
-      <c r="A24" s="9"/>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9"/>
-      <c r="D24" s="29"/>
-      <c r="E24" s="9"/>
-      <c r="F24" s="9"/>
-      <c r="G24" s="28"/>
-      <c r="H24" s="28"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="28"/>
+      <c r="A24" s="17"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="30"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="37"/>
+      <c r="H24" s="37"/>
+      <c r="I24" s="37"/>
+      <c r="J24" s="37"/>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="7">
         <v>17</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
-      <c r="G25" s="30" t="s">
-        <v>99</v>
-      </c>
-      <c r="H25" s="31"/>
-      <c r="I25" s="31"/>
-      <c r="J25" s="32"/>
+      <c r="G25" s="31" t="s">
+        <v>96</v>
+      </c>
+      <c r="H25" s="32"/>
+      <c r="I25" s="32"/>
+      <c r="J25" s="33"/>
     </row>
     <row r="26" spans="1:10" ht="16.5" customHeight="1">
-      <c r="A26" s="9">
+      <c r="A26" s="17">
         <v>18</v>
       </c>
-      <c r="B26" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="H26" s="24"/>
-      <c r="I26" s="24"/>
-      <c r="J26" s="24"/>
+      <c r="B26" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+      <c r="J26" s="38"/>
     </row>
     <row r="27" spans="1:10">
-      <c r="A27" s="9"/>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9"/>
-      <c r="D27" s="9"/>
-      <c r="E27" s="9"/>
-      <c r="F27" s="9"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
-      <c r="I27" s="24"/>
-      <c r="J27" s="24"/>
+      <c r="A27" s="17"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="17"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
+      <c r="J27" s="38"/>
     </row>
     <row r="28" spans="1:10">
-      <c r="A28" s="9"/>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="9"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
+      <c r="A28" s="17"/>
+      <c r="B28" s="17"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+      <c r="J28" s="38"/>
     </row>
     <row r="29" spans="1:10">
-      <c r="A29" s="9"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="9"/>
-      <c r="D29" s="9"/>
-      <c r="E29" s="9"/>
-      <c r="F29" s="9"/>
-      <c r="G29" s="24"/>
-      <c r="H29" s="24"/>
-      <c r="I29" s="24"/>
-      <c r="J29" s="24"/>
+      <c r="A29" s="17"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
+      <c r="J29" s="38"/>
     </row>
     <row r="30" spans="1:10" ht="17.25">
       <c r="A30" s="7">
         <v>19</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E30" s="3"/>
       <c r="F30" s="3"/>
-      <c r="G30" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="H30" s="26"/>
-      <c r="I30" s="26"/>
-      <c r="J30" s="27"/>
+      <c r="G30" s="27" t="s">
+        <v>99</v>
+      </c>
+      <c r="H30" s="28"/>
+      <c r="I30" s="28"/>
+      <c r="J30" s="29"/>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="3">
         <v>20</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>37</v>
+        <v>98</v>
       </c>
       <c r="E31" s="3"/>
       <c r="F31" s="3"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="26"/>
-      <c r="I31" s="26"/>
-      <c r="J31" s="27"/>
+      <c r="G31" s="27" t="s">
+        <v>132</v>
+      </c>
+      <c r="H31" s="28"/>
+      <c r="I31" s="28"/>
+      <c r="J31" s="29"/>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="7">
         <v>21</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E32" s="4"/>
       <c r="F32" s="4"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="26"/>
-      <c r="I32" s="26"/>
-      <c r="J32" s="27"/>
+      <c r="G32" s="27"/>
+      <c r="H32" s="28"/>
+      <c r="I32" s="28"/>
+      <c r="J32" s="29"/>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="3">
         <v>22</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E33" s="4"/>
       <c r="F33" s="4"/>
-      <c r="G33" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="H33" s="26"/>
-      <c r="I33" s="26"/>
-      <c r="J33" s="27"/>
+      <c r="G33" s="27" t="s">
+        <v>101</v>
+      </c>
+      <c r="H33" s="28"/>
+      <c r="I33" s="28"/>
+      <c r="J33" s="29"/>
     </row>
     <row r="34" spans="1:10">
       <c r="A34" s="3">
         <v>23</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E34" s="4"/>
       <c r="F34" s="4"/>
-      <c r="G34" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="H34" s="26"/>
-      <c r="I34" s="26"/>
-      <c r="J34" s="27"/>
+      <c r="G34" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="H34" s="28"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="29"/>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" s="11">
+        <v>24</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="27"/>
+      <c r="H35" s="28"/>
+      <c r="I35" s="28"/>
+      <c r="J35" s="29"/>
     </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="48">
+    <mergeCell ref="G35:J35"/>
     <mergeCell ref="G21:J21"/>
     <mergeCell ref="G10:J10"/>
     <mergeCell ref="A2:J3"/>
@@ -2267,13 +2284,13 @@
     <mergeCell ref="F26:F29"/>
     <mergeCell ref="G22:J22"/>
     <mergeCell ref="G23:J24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G26:J29"/>
     <mergeCell ref="A23:A24"/>
     <mergeCell ref="B23:B24"/>
     <mergeCell ref="C23:C24"/>
     <mergeCell ref="D23:D24"/>
     <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G26:J29"/>
     <mergeCell ref="G31:J31"/>
     <mergeCell ref="G30:J30"/>
     <mergeCell ref="G34:J34"/>
@@ -2300,136 +2317,136 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="19"/>
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
+      <c r="A3" s="22"/>
+      <c r="B3" s="22"/>
+      <c r="C3" s="22"/>
+      <c r="D3" s="22"/>
+      <c r="E3" s="22"/>
+      <c r="F3" s="22"/>
+      <c r="G3" s="22"/>
+      <c r="H3" s="22"/>
+      <c r="I3" s="22"/>
+      <c r="J3" s="22"/>
     </row>
     <row r="4" spans="1:10">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="21"/>
-      <c r="C4" s="22" t="s">
-        <v>109</v>
-      </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="20" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="25" t="s">
+        <v>104</v>
+      </c>
+      <c r="D4" s="26"/>
+      <c r="E4" s="26"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22" t="s">
+      <c r="H4" s="24"/>
+      <c r="I4" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="21"/>
+      <c r="J4" s="24"/>
     </row>
     <row r="5" spans="1:10">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="15" t="s">
-        <v>110</v>
-      </c>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="13" t="s">
+      <c r="B5" s="16"/>
+      <c r="C5" s="18" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="16"/>
+      <c r="G5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="15" t="s">
+      <c r="H5" s="16"/>
+      <c r="I5" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="14"/>
+      <c r="J5" s="16"/>
     </row>
     <row r="6" spans="1:10">
-      <c r="A6" s="36" t="s">
+      <c r="A6" s="39" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="37" t="s">
-        <v>111</v>
-      </c>
-      <c r="D6" s="38"/>
-      <c r="E6" s="38"/>
-      <c r="F6" s="38"/>
-      <c r="G6" s="38"/>
-      <c r="H6" s="38"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="39"/>
+      <c r="B6" s="14"/>
+      <c r="C6" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
+      <c r="I6" s="41"/>
+      <c r="J6" s="42"/>
     </row>
     <row r="7" spans="1:10">
-      <c r="A7" s="40" t="s">
+      <c r="A7" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="40" t="s">
-        <v>105</v>
-      </c>
-      <c r="C7" s="40" t="s">
+      <c r="B7" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="D7" s="40" t="s">
+      <c r="D7" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="40" t="s">
+      <c r="E7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="40" t="s">
+      <c r="F7" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="G7" s="41" t="s">
+      <c r="G7" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="H7" s="42"/>
-      <c r="I7" s="42"/>
-      <c r="J7" s="42"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="8">
         <v>1</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E8" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="F8" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="25"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="29"/>
     </row>
     <row r="9" spans="1:10" ht="17.25">
       <c r="A9" s="8">
@@ -2439,121 +2456,121 @@
         <v>15</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="F9" s="43" t="s">
-        <v>113</v>
-      </c>
-      <c r="G9" s="25"/>
-      <c r="H9" s="26"/>
-      <c r="I9" s="26"/>
-      <c r="J9" s="27"/>
+        <v>39</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="G9" s="27"/>
+      <c r="H9" s="28"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="29"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10" s="8">
         <v>3</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="26"/>
-      <c r="I10" s="26"/>
-      <c r="J10" s="27"/>
+      <c r="G10" s="27"/>
+      <c r="H10" s="28"/>
+      <c r="I10" s="28"/>
+      <c r="J10" s="29"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11" s="8">
         <v>4</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="26"/>
-      <c r="I11" s="26"/>
-      <c r="J11" s="27"/>
+      <c r="G11" s="27"/>
+      <c r="H11" s="28"/>
+      <c r="I11" s="28"/>
+      <c r="J11" s="29"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="8">
         <v>5</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
-      <c r="G12" s="25"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="28"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="29"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13" s="8">
         <v>6</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="26"/>
-      <c r="I13" s="26"/>
-      <c r="J13" s="27"/>
+      <c r="G13" s="27"/>
+      <c r="H13" s="28"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="29"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" s="8">
         <v>7</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="26"/>
-      <c r="J14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="29"/>
     </row>
   </sheetData>
   <mergeCells count="19">
@@ -2567,15 +2584,15 @@
     <mergeCell ref="G8:J8"/>
     <mergeCell ref="G9:J9"/>
     <mergeCell ref="G10:J10"/>
+    <mergeCell ref="A5:B5"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
     <mergeCell ref="A2:J3"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="C4:F4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:J4"/>
-    <mergeCell ref="A5:B5"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>